<commit_message>
Modelo de 10 nodos con 0% GAP
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -1908,20 +1908,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[8, 6, 7, 8]</t>
+          <t>[8, 2, 1, 8]</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1015</v>
+        <v>3357</v>
       </c>
       <c r="E10" t="n">
-        <v>76.20999999999999</v>
+        <v>70.16</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>996.5792246608871</v>
+        <v>3338.579224660887</v>
       </c>
       <c r="H10" t="n">
         <v>216.9179260871245</v>
@@ -2034,7 +2034,7 @@
         <v>1</v>
       </c>
       <c r="AL10" t="n">
-        <v>69.7646708370569</v>
+        <v>0</v>
       </c>
       <c r="AM10" t="n">
         <v>0</v>
@@ -2052,7 +2052,7 @@
         <v>0</v>
       </c>
       <c r="AR10" t="n">
-        <v>70.31339813342606</v>
+        <v>0.5487272963691788</v>
       </c>
     </row>
     <row r="11">
@@ -2300,7 +2300,7 @@
         <v>1094.8</v>
       </c>
       <c r="D2" t="n">
-        <v>860.6</v>
+        <v>1094.8</v>
       </c>
       <c r="E2" t="n">
         <v>580.6</v>
@@ -2318,13 +2318,13 @@
         <v>874.4</v>
       </c>
       <c r="J2" t="n">
-        <v>632.9528086185455</v>
+        <v>641.6470177173615</v>
       </c>
       <c r="K2" t="n">
-        <v>6.97646708370569</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>6.508765095952453</v>
+        <v>-0.4677019877532351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prueba inicial nuevo servidor
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -681,10 +681,10 @@
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1913.299455076057</v>
+        <v>2011.31602136959</v>
       </c>
       <c r="I2" t="n">
-        <v>231.1086937254513</v>
+        <v>216.126539257865</v>
       </c>
       <c r="J2" t="n">
         <v>100</v>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="AS2" t="n">
-        <v>2.581494140730317</v>
+        <v>-2.409166057514771</v>
       </c>
     </row>
     <row r="3">
@@ -840,10 +840,10 @@
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>1586.394183838217</v>
+        <v>1586.986222695625</v>
       </c>
       <c r="I3" t="n">
-        <v>235.2986933881506</v>
+        <v>252.3813434255695</v>
       </c>
       <c r="J3" t="n">
         <v>100</v>
@@ -971,7 +971,7 @@
         <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>-0.9798971252843576</v>
+        <v>-1.017582603158814</v>
       </c>
     </row>
     <row r="4">
@@ -999,10 +999,10 @@
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>2783.234332978707</v>
+        <v>2760.278831402291</v>
       </c>
       <c r="I4" t="n">
-        <v>173.9904637917831</v>
+        <v>231.079398263637</v>
       </c>
       <c r="J4" t="n">
         <v>100</v>
@@ -1130,7 +1130,7 @@
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.8113209914929707</v>
+        <v>1.62940729143653</v>
       </c>
     </row>
     <row r="5">
@@ -1158,10 +1158,10 @@
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1257.826492502043</v>
+        <v>1265.831701624215</v>
       </c>
       <c r="I5" t="n">
-        <v>267.586202055649</v>
+        <v>220.9660711017475</v>
       </c>
       <c r="J5" t="n">
         <v>100</v>
@@ -1289,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>1.809016978763247</v>
+        <v>1.184098233862968</v>
       </c>
     </row>
     <row r="6">
@@ -1317,10 +1317,10 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1136.974121227615</v>
+        <v>1073.385617373551</v>
       </c>
       <c r="I6" t="n">
-        <v>199.0611795127753</v>
+        <v>265.1612341226595</v>
       </c>
       <c r="J6" t="n">
         <v>100</v>
@@ -1448,7 +1448,7 @@
         <v>0</v>
       </c>
       <c r="AS6" t="n">
-        <v>-5.275381595149526</v>
+        <v>0.6124428357823372</v>
       </c>
     </row>
     <row r="7">
@@ -1476,10 +1476,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>834.2347350938169</v>
+        <v>789.5176716168876</v>
       </c>
       <c r="I7" t="n">
-        <v>225.382075148047</v>
+        <v>238.3649227196198</v>
       </c>
       <c r="J7" t="n">
         <v>100</v>
@@ -1607,7 +1607,7 @@
         <v>0</v>
       </c>
       <c r="AS7" t="n">
-        <v>-7.782265515997013</v>
+        <v>-2.004867133964804</v>
       </c>
     </row>
     <row r="8">
@@ -1635,10 +1635,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>2002.01364429514</v>
+        <v>1960.085395744783</v>
       </c>
       <c r="I8" t="n">
-        <v>239.0863568109169</v>
+        <v>220.8876706135575</v>
       </c>
       <c r="J8" t="n">
         <v>100</v>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="AS8" t="n">
-        <v>-1.9355216036222</v>
+        <v>0.1993179356017034</v>
       </c>
     </row>
     <row r="9">
@@ -1794,10 +1794,10 @@
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>2802.605191163997</v>
+        <v>2782.696105400663</v>
       </c>
       <c r="I9" t="n">
-        <v>224.0429602876613</v>
+        <v>216.7454332700319</v>
       </c>
       <c r="J9" t="n">
         <v>100</v>
@@ -1925,7 +1925,7 @@
         <v>5.72655690765927</v>
       </c>
       <c r="AS9" t="n">
-        <v>-0.3079882306369723</v>
+        <v>0.4045774731330233</v>
       </c>
     </row>
     <row r="10">
@@ -1953,10 +1953,10 @@
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>1764.620014476918</v>
+        <v>1887.570935340693</v>
       </c>
       <c r="I10" t="n">
-        <v>218.9960015891271</v>
+        <v>204.1290610494041</v>
       </c>
       <c r="J10" t="n">
         <v>100</v>
@@ -2084,7 +2084,7 @@
         <v>0</v>
       </c>
       <c r="AS10" t="n">
-        <v>5.836712141039572</v>
+        <v>-0.7241694418726154</v>
       </c>
     </row>
     <row r="11">
@@ -2112,10 +2112,10 @@
         <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>-4038.957526093422</v>
+        <v>-4109.634212016557</v>
       </c>
       <c r="I11" t="n">
-        <v>223.3432108199351</v>
+        <v>187.0689967411276</v>
       </c>
       <c r="J11" t="n">
         <v>100</v>
@@ -2243,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>-0.07527149694650978</v>
+        <v>1.673285799518983</v>
       </c>
     </row>
   </sheetData>
@@ -2353,13 +2353,13 @@
         <v>1190.6</v>
       </c>
       <c r="J2" t="n">
-        <v>705.8038966655731</v>
+        <v>978.8405251502991</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.5317781315610473</v>
+        <v>-0.04526556671754604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización a días dinámicos dentro del episodio
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS11"/>
+  <dimension ref="A1:AX11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,190 +467,215 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>DRL Real Route</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Reward</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Duration</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Valid</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>DRL Stoch Mean</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>DRL Stoch Std</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>DRL Stoch Valid%</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>MIP Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MIP Route</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MIP Reward</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MIP Duration</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>MIP Valid</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Route</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Reward</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Duration</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Valid</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>2Opt Route</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>2Opt Reward</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>2Opt Duration</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>2Opt Valid</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>GA Status</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>GA Route</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>GA Reward</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>GA Duration</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>GA Valid</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>LNS Status</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>LNS Route</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LNS Reward</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>LNS Duration</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LNS Valid</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>DRL Gap (%)</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Gap (%)</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Gap (%)</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>2Opt Gap (%)</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>GA Gap (%)</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>LNS Gap (%)</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Gap (%)</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>DRL Stoch Gap (%)</t>
         </is>
@@ -680,139 +705,156 @@
       <c r="G2" t="b">
         <v>1</v>
       </c>
-      <c r="H2" t="n">
-        <v>2011.31602136959</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
       </c>
       <c r="I2" t="n">
-        <v>216.126539257865</v>
+        <v>2041</v>
       </c>
       <c r="J2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1988.392767760048</v>
+      </c>
+      <c r="M2" t="n">
+        <v>204.2786360744227</v>
+      </c>
+      <c r="N2" t="n">
         <v>100</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="Q2" t="n">
         <v>1964</v>
       </c>
-      <c r="N2" t="n">
+      <c r="R2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="O2" t="b">
-        <v>1</v>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="S2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="U2" t="n">
         <v>1735</v>
       </c>
-      <c r="R2" t="n">
+      <c r="V2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="S2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="W2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="U2" t="n">
+      <c r="Y2" t="n">
         <v>1964</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Z2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="W2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="Z2" t="n">
+      <c r="AD2" t="n">
         <v>1964</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AE2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AB2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
         <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="AE2" t="n">
+      <c r="AI2" t="n">
         <v>1735</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AJ2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="AG2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AK2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AN2" t="n">
         <v>1964</v>
       </c>
-      <c r="AK2" t="n">
+      <c r="AO2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AL2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN2" t="n">
+      <c r="AP2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>-3.920570264765784</v>
+      </c>
+      <c r="AS2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AO2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="n">
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AR2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>-2.409166057514771</v>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>-1.241994285134847</v>
       </c>
     </row>
     <row r="3">
@@ -839,139 +881,156 @@
       <c r="G3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" t="n">
-        <v>1586.986222695625</v>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
       </c>
       <c r="I3" t="n">
-        <v>252.3813434255695</v>
+        <v>1656</v>
       </c>
       <c r="J3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1582.223467129861</v>
+      </c>
+      <c r="M3" t="n">
+        <v>234.1582207210608</v>
+      </c>
+      <c r="N3" t="n">
         <v>100</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="Q3" t="n">
         <v>1571</v>
       </c>
-      <c r="N3" t="n">
+      <c r="R3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="O3" t="b">
-        <v>1</v>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="S3" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="U3" t="n">
         <v>-773</v>
       </c>
-      <c r="R3" t="n">
+      <c r="V3" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="S3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t>[1, 8, 2, 1]</t>
         </is>
       </c>
-      <c r="U3" t="n">
+      <c r="Y3" t="n">
         <v>-669</v>
       </c>
-      <c r="V3" t="n">
+      <c r="Z3" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="W3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>1571</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AB3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="AE3" t="n">
+      <c r="AI3" t="n">
         <v>-773</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AJ3" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AG3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AK3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AN3" t="n">
         <v>1571</v>
       </c>
-      <c r="AK3" t="n">
+      <c r="AO3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AL3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN3" t="n">
+      <c r="AP3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>-5.410566518141311</v>
+      </c>
+      <c r="AS3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AT3" t="n">
         <v>142.5843411839593</v>
       </c>
-      <c r="AP3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ3" t="n">
+      <c r="AU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AR3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>-1.017582603158814</v>
+      <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>-0.7144154761209827</v>
       </c>
     </row>
     <row r="4">
@@ -998,139 +1057,156 @@
       <c r="G4" t="b">
         <v>1</v>
       </c>
-      <c r="H4" t="n">
-        <v>2760.278831402291</v>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[2, 6, 8, 2]</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>231.079398263637</v>
+        <v>2486</v>
       </c>
       <c r="J4" t="n">
+        <v>72.44731374037281</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2869.710009649785</v>
+      </c>
+      <c r="M4" t="n">
+        <v>239.9112793821178</v>
+      </c>
+      <c r="N4" t="n">
         <v>100</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="Q4" t="n">
         <v>2806</v>
       </c>
-      <c r="N4" t="n">
+      <c r="R4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="S4" t="b">
+        <v>1</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="U4" t="n">
         <v>976</v>
       </c>
-      <c r="R4" t="n">
+      <c r="V4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="S4" t="b">
-        <v>1</v>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="U4" t="n">
+      <c r="Y4" t="n">
         <v>2806</v>
       </c>
-      <c r="V4" t="n">
+      <c r="Z4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="W4" t="b">
-        <v>1</v>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AA4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="Z4" t="n">
+      <c r="AD4" t="n">
         <v>2806</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AE4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AB4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AF4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AE4" t="n">
+      <c r="AI4" t="n">
         <v>976</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AJ4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="AG4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AK4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AN4" t="n">
         <v>2806</v>
       </c>
-      <c r="AK4" t="n">
+      <c r="AO4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AL4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN4" t="n">
+      <c r="AP4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>11.40413399857448</v>
+      </c>
+      <c r="AS4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AO4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AR4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>1.62940729143653</v>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>-2.27049214717695</v>
       </c>
     </row>
     <row r="5">
@@ -1157,33 +1233,33 @@
       <c r="G5" t="b">
         <v>1</v>
       </c>
-      <c r="H5" t="n">
-        <v>1265.831701624215</v>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[3, 4, 3]</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>220.9660711017475</v>
+        <v>1344</v>
       </c>
       <c r="J5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1235.411193022208</v>
+      </c>
+      <c r="M5" t="n">
+        <v>233.587028357313</v>
+      </c>
+      <c r="N5" t="n">
         <v>100</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>[3, 4, 3]</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>1281</v>
-      </c>
-      <c r="N5" t="n">
-        <v>40.68356024804761</v>
-      </c>
-      <c r="O5" t="b">
-        <v>1</v>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1215,81 +1291,98 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
+      <c r="Y5" t="n">
+        <v>1281</v>
+      </c>
       <c r="Z5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="AD5" t="n">
         <v>1281</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AE5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AB5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AE5" t="n">
+      <c r="AI5" t="n">
         <v>1281</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AJ5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AG5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AK5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AN5" t="n">
         <v>1281</v>
       </c>
-      <c r="AK5" t="n">
+      <c r="AO5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AL5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>0</v>
+      <c r="AP5" t="b">
+        <v>1</v>
       </c>
       <c r="AQ5" t="n">
         <v>0</v>
       </c>
       <c r="AR5" t="n">
-        <v>0</v>
+        <v>-4.918032786885246</v>
       </c>
       <c r="AS5" t="n">
-        <v>1.184098233862968</v>
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>3.558845197329554</v>
       </c>
     </row>
     <row r="6">
@@ -1316,33 +1409,33 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" t="n">
-        <v>1073.385617373551</v>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[4, 3, 4]</t>
+        </is>
       </c>
       <c r="I6" t="n">
-        <v>265.1612341226595</v>
+        <v>1281</v>
       </c>
       <c r="J6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1086.430256826657</v>
+      </c>
+      <c r="M6" t="n">
+        <v>255.4162398248407</v>
+      </c>
+      <c r="N6" t="n">
         <v>100</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>[4, 3, 4]</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
-        <v>1080</v>
-      </c>
-      <c r="N6" t="n">
-        <v>40.68356024804761</v>
-      </c>
-      <c r="O6" t="b">
-        <v>1</v>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1374,81 +1467,98 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
+      <c r="Y6" t="n">
+        <v>1080</v>
+      </c>
       <c r="Z6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="AD6" t="n">
         <v>1080</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AE6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AB6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AF6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AE6" t="n">
+      <c r="AI6" t="n">
         <v>1080</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AJ6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AG6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AK6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AN6" t="n">
         <v>1080</v>
       </c>
-      <c r="AK6" t="n">
+      <c r="AO6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AL6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>0</v>
+      <c r="AP6" t="b">
+        <v>1</v>
       </c>
       <c r="AQ6" t="n">
         <v>0</v>
       </c>
       <c r="AR6" t="n">
-        <v>0</v>
+        <v>-18.61111111111111</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.6124428357823372</v>
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>-0.5953941506163574</v>
       </c>
     </row>
     <row r="7">
@@ -1475,33 +1585,33 @@
       <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="H7" t="n">
-        <v>789.5176716168876</v>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[5, 3, 5]</t>
+        </is>
       </c>
       <c r="I7" t="n">
-        <v>238.3649227196198</v>
+        <v>781</v>
       </c>
       <c r="J7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>725.9777883330827</v>
+      </c>
+      <c r="M7" t="n">
+        <v>216.9870634967322</v>
+      </c>
+      <c r="N7" t="n">
         <v>100</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>[5, 3, 5]</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>774</v>
-      </c>
-      <c r="N7" t="n">
-        <v>48.69171070169158</v>
-      </c>
-      <c r="O7" t="b">
-        <v>1</v>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1533,81 +1643,98 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
+      <c r="Y7" t="n">
+        <v>774</v>
+      </c>
       <c r="Z7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="AD7" t="n">
         <v>774</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AE7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AB7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AF7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AE7" t="n">
+      <c r="AI7" t="n">
         <v>774</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AJ7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AG7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
+      <c r="AK7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AN7" t="n">
         <v>774</v>
       </c>
-      <c r="AK7" t="n">
+      <c r="AO7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AL7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>0</v>
+      <c r="AP7" t="b">
+        <v>1</v>
       </c>
       <c r="AQ7" t="n">
         <v>0</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>-0.9043927648578811</v>
       </c>
       <c r="AS7" t="n">
-        <v>-2.004867133964804</v>
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>6.20442011200482</v>
       </c>
     </row>
     <row r="8">
@@ -1634,33 +1761,33 @@
       <c r="G8" t="b">
         <v>1</v>
       </c>
-      <c r="H8" t="n">
-        <v>1960.085395744783</v>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
       </c>
       <c r="I8" t="n">
-        <v>220.8876706135575</v>
+        <v>2021</v>
       </c>
       <c r="J8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1941.713082628688</v>
+      </c>
+      <c r="M8" t="n">
+        <v>223.9113465054168</v>
+      </c>
+      <c r="N8" t="n">
         <v>100</v>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>[6, 0, 1, 6]</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>1964</v>
-      </c>
-      <c r="N8" t="n">
-        <v>76.7052345103569</v>
-      </c>
-      <c r="O8" t="b">
-        <v>1</v>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
@@ -1692,81 +1819,98 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
+      <c r="Y8" t="n">
+        <v>1964</v>
+      </c>
       <c r="Z8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>[6, 0, 1, 6]</t>
+        </is>
+      </c>
+      <c r="AD8" t="n">
         <v>1964</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AE8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AB8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD8" t="inlineStr">
+      <c r="AF8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="AE8" t="n">
+      <c r="AI8" t="n">
         <v>1964</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AJ8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AG8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
+      <c r="AK8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AN8" t="n">
         <v>1964</v>
       </c>
-      <c r="AK8" t="n">
+      <c r="AO8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AL8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="n">
-        <v>0</v>
+      <c r="AP8" t="b">
+        <v>1</v>
       </c>
       <c r="AQ8" t="n">
         <v>0</v>
       </c>
       <c r="AR8" t="n">
-        <v>0</v>
+        <v>-2.90224032586558</v>
       </c>
       <c r="AS8" t="n">
-        <v>0.1993179356017034</v>
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>1.134771760250115</v>
       </c>
     </row>
     <row r="9">
@@ -1793,44 +1937,44 @@
       <c r="G9" t="b">
         <v>1</v>
       </c>
-      <c r="H9" t="n">
-        <v>2782.696105400663</v>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[7, 8, 7]</t>
+        </is>
       </c>
       <c r="I9" t="n">
-        <v>216.7454332700319</v>
+        <v>2291</v>
       </c>
       <c r="J9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2820.597360020625</v>
+      </c>
+      <c r="M9" t="n">
+        <v>264.705656476628</v>
+      </c>
+      <c r="N9" t="n">
         <v>100</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="Q9" t="n">
         <v>2794</v>
       </c>
-      <c r="N9" t="n">
+      <c r="R9" t="n">
         <v>72.81063071208843</v>
-      </c>
-      <c r="O9" t="b">
-        <v>1</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>[7, 8, 6, 7]</t>
-        </is>
-      </c>
-      <c r="Q9" t="n">
-        <v>2634</v>
-      </c>
-      <c r="R9" t="n">
-        <v>76.25197526044872</v>
       </c>
       <c r="S9" t="b">
         <v>1</v>
@@ -1851,81 +1995,98 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
+      <c r="Y9" t="n">
+        <v>2634</v>
+      </c>
       <c r="Z9" t="n">
+        <v>76.25197526044872</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>[7, 8, 6, 7]</t>
+        </is>
+      </c>
+      <c r="AD9" t="n">
         <v>2634</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AE9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AB9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
+      <c r="AF9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="AE9" t="n">
+      <c r="AI9" t="n">
         <v>2634</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AJ9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AG9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
+      <c r="AK9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AN9" t="n">
         <v>2634</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AO9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AL9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN9" t="n">
+      <c r="AP9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>18.00286327845383</v>
+      </c>
+      <c r="AS9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="AT9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="AU9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="AV9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="AW9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AS9" t="n">
-        <v>0.4045774731330233</v>
+      <c r="AX9" t="n">
+        <v>-0.9519455984475761</v>
       </c>
     </row>
     <row r="10">
@@ -1952,33 +2113,33 @@
       <c r="G10" t="b">
         <v>1</v>
       </c>
-      <c r="H10" t="n">
-        <v>1887.570935340693</v>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
       </c>
       <c r="I10" t="n">
-        <v>204.1290610494041</v>
+        <v>1707</v>
       </c>
       <c r="J10" t="n">
+        <v>70.15987690240341</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1846.929181506918</v>
+      </c>
+      <c r="M10" t="n">
+        <v>264.658784780783</v>
+      </c>
+      <c r="N10" t="n">
         <v>100</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>[8, 1, 2, 8]</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>1874</v>
-      </c>
-      <c r="N10" t="n">
-        <v>70.15987690240341</v>
-      </c>
-      <c r="O10" t="b">
-        <v>1</v>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
@@ -1989,7 +2150,7 @@
         <v>1874</v>
       </c>
       <c r="R10" t="n">
-        <v>70.15987690240343</v>
+        <v>70.15987690240341</v>
       </c>
       <c r="S10" t="b">
         <v>1</v>
@@ -2010,81 +2171,98 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
+      <c r="Y10" t="n">
+        <v>1874</v>
+      </c>
       <c r="Z10" t="n">
+        <v>70.15987690240343</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>[8, 1, 2, 8]</t>
+        </is>
+      </c>
+      <c r="AD10" t="n">
         <v>1874</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AE10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AB10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AF10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="AE10" t="n">
+      <c r="AI10" t="n">
         <v>1874</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AJ10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AG10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr">
+      <c r="AK10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AN10" t="n">
         <v>1874</v>
       </c>
-      <c r="AK10" t="n">
+      <c r="AO10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AL10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM10" t="n">
+      <c r="AP10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AQ10" t="n">
         <v>1.387406616862326</v>
       </c>
-      <c r="AN10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>0</v>
-      </c>
       <c r="AR10" t="n">
-        <v>0</v>
+        <v>8.911419423692637</v>
       </c>
       <c r="AS10" t="n">
-        <v>-0.7241694418726154</v>
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>1.44454741158391</v>
       </c>
     </row>
     <row r="11">
@@ -2111,33 +2289,33 @@
       <c r="G11" t="b">
         <v>1</v>
       </c>
-      <c r="H11" t="n">
-        <v>-4109.634212016557</v>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>[9, 2, 9]</t>
+        </is>
       </c>
       <c r="I11" t="n">
-        <v>187.0689967411276</v>
+        <v>-4042</v>
       </c>
       <c r="J11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-4045.336492465923</v>
+      </c>
+      <c r="M11" t="n">
+        <v>231.2754224150323</v>
+      </c>
+      <c r="N11" t="n">
         <v>100</v>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>[9, 2, 9]</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>-4042</v>
-      </c>
-      <c r="N11" t="n">
-        <v>64.70237352474922</v>
-      </c>
-      <c r="O11" t="b">
-        <v>1</v>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
@@ -2169,72 +2347,74 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
+      <c r="Y11" t="n">
+        <v>-4042</v>
+      </c>
       <c r="Z11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="AD11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AE11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AB11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
+      <c r="AF11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AE11" t="n">
+      <c r="AI11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AJ11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AG11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AI11" t="inlineStr">
+      <c r="AK11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AN11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AK11" t="n">
+      <c r="AO11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AL11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>0</v>
+      <c r="AP11" t="b">
+        <v>1</v>
       </c>
       <c r="AQ11" t="n">
         <v>0</v>
@@ -2243,7 +2423,22 @@
         <v>0</v>
       </c>
       <c r="AS11" t="n">
-        <v>1.673285799518983</v>
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0.08254558302629081</v>
       </c>
     </row>
   </sheetData>
@@ -2353,13 +2548,13 @@
         <v>1190.6</v>
       </c>
       <c r="J2" t="n">
-        <v>978.8405251502991</v>
+        <v>944.7880446910858</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.04526556671754604</v>
+        <v>0.6650888406697978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicion de señales de mercado
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -720,10 +720,10 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1988.392767760048</v>
+        <v>1927.120138742865</v>
       </c>
       <c r="M2" t="n">
-        <v>204.2786360744227</v>
+        <v>187.9019456485501</v>
       </c>
       <c r="N2" t="n">
         <v>100</v>
@@ -854,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="AX2" t="n">
-        <v>-1.241994285134847</v>
+        <v>1.8777933430313</v>
       </c>
     </row>
     <row r="3">
@@ -896,10 +896,10 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1582.223467129861</v>
+        <v>1562.868810989135</v>
       </c>
       <c r="M3" t="n">
-        <v>234.1582207210608</v>
+        <v>239.3835359491156</v>
       </c>
       <c r="N3" t="n">
         <v>100</v>
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="AX3" t="n">
-        <v>-0.7144154761209827</v>
+        <v>0.5175804589983942</v>
       </c>
     </row>
     <row r="4">
@@ -1072,10 +1072,10 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2869.710009649785</v>
+        <v>2819.378375257139</v>
       </c>
       <c r="M4" t="n">
-        <v>239.9112793821178</v>
+        <v>205.3565369082927</v>
       </c>
       <c r="N4" t="n">
         <v>100</v>
@@ -1206,7 +1206,7 @@
         <v>0</v>
       </c>
       <c r="AX4" t="n">
-        <v>-2.27049214717695</v>
+        <v>-0.4767774503613308</v>
       </c>
     </row>
     <row r="5">
@@ -1248,10 +1248,10 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>1235.411193022208</v>
+        <v>1274.754116106943</v>
       </c>
       <c r="M5" t="n">
-        <v>233.587028357313</v>
+        <v>229.4779984606443</v>
       </c>
       <c r="N5" t="n">
         <v>100</v>
@@ -1382,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="AX5" t="n">
-        <v>3.558845197329554</v>
+        <v>0.4875787582402206</v>
       </c>
     </row>
     <row r="6">
@@ -1424,10 +1424,10 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>1086.430256826657</v>
+        <v>1106.777517792156</v>
       </c>
       <c r="M6" t="n">
-        <v>255.4162398248407</v>
+        <v>227.9874804161272</v>
       </c>
       <c r="N6" t="n">
         <v>100</v>
@@ -1558,7 +1558,7 @@
         <v>0</v>
       </c>
       <c r="AX6" t="n">
-        <v>-0.5953941506163574</v>
+        <v>-2.479399795570021</v>
       </c>
     </row>
     <row r="7">
@@ -1600,10 +1600,10 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>725.9777883330827</v>
+        <v>733.5806640148237</v>
       </c>
       <c r="M7" t="n">
-        <v>216.9870634967322</v>
+        <v>167.5705297236776</v>
       </c>
       <c r="N7" t="n">
         <v>100</v>
@@ -1734,7 +1734,7 @@
         <v>0</v>
       </c>
       <c r="AX7" t="n">
-        <v>6.20442011200482</v>
+        <v>5.222136432193321</v>
       </c>
     </row>
     <row r="8">
@@ -1776,10 +1776,10 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>1941.713082628688</v>
+        <v>1992.088721972067</v>
       </c>
       <c r="M8" t="n">
-        <v>223.9113465054168</v>
+        <v>218.4144072876398</v>
       </c>
       <c r="N8" t="n">
         <v>100</v>
@@ -1910,7 +1910,7 @@
         <v>0</v>
       </c>
       <c r="AX8" t="n">
-        <v>1.134771760250115</v>
+        <v>-1.430179326479995</v>
       </c>
     </row>
     <row r="9">
@@ -1952,10 +1952,10 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>2820.597360020625</v>
+        <v>2773.479890320478</v>
       </c>
       <c r="M9" t="n">
-        <v>264.705656476628</v>
+        <v>242.7141642794886</v>
       </c>
       <c r="N9" t="n">
         <v>100</v>
@@ -2086,7 +2086,7 @@
         <v>5.72655690765927</v>
       </c>
       <c r="AX9" t="n">
-        <v>-0.9519455984475761</v>
+        <v>0.7344348489449604</v>
       </c>
     </row>
     <row r="10">
@@ -2128,10 +2128,10 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1846.929181506918</v>
+        <v>1801.844142827736</v>
       </c>
       <c r="M10" t="n">
-        <v>264.658784780783</v>
+        <v>231.3565177255371</v>
       </c>
       <c r="N10" t="n">
         <v>100</v>
@@ -2262,7 +2262,7 @@
         <v>0</v>
       </c>
       <c r="AX10" t="n">
-        <v>1.44454741158391</v>
+        <v>3.850365911006627</v>
       </c>
     </row>
     <row r="11">
@@ -2304,10 +2304,10 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>-4045.336492465923</v>
+        <v>-4050.96728546096</v>
       </c>
       <c r="M11" t="n">
-        <v>231.2754224150323</v>
+        <v>235.0732453317911</v>
       </c>
       <c r="N11" t="n">
         <v>100</v>
@@ -2438,7 +2438,7 @@
         <v>0</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.08254558302629081</v>
+        <v>0.2218526833488442</v>
       </c>
     </row>
   </sheetData>
@@ -2548,13 +2548,13 @@
         <v>1190.6</v>
       </c>
       <c r="J2" t="n">
-        <v>944.7880446910858</v>
+        <v>1021.136117458344</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>
       </c>
       <c r="L2" t="n">
-        <v>0.6650888406697978</v>
+        <v>0.8525385863352319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Separación ruido de train y eval
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX11"/>
+  <dimension ref="A1:AZ11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,185 +497,195 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>DRL Stoch CVaR</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Stoch P10</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>DRL Stoch Valid%</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MIP Status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MIP Route</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>MIP Reward</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MIP Duration</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MIP Valid</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Route</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Reward</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Duration</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Valid</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>2Opt Route</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>2Opt Reward</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>2Opt Duration</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>2Opt Valid</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>GA Status</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>GA Route</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>GA Reward</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>GA Duration</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>GA Valid</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LNS Status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>LNS Route</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LNS Reward</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>LNS Duration</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>LNS Valid</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>DRL Gap (%)</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Gap (%)</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Heuristic Gap (%)</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>2Opt Gap (%)</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>GA Gap (%)</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>LNS Gap (%)</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Gap (%)</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>DRL Stoch Gap (%)</t>
         </is>
@@ -720,141 +730,147 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>1927.120138742865</v>
+        <v>2107.161117247363</v>
       </c>
       <c r="M2" t="n">
-        <v>187.9019456485501</v>
+        <v>316.4903617400911</v>
       </c>
       <c r="N2" t="n">
+        <v>1714.415180865755</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1716.558778331066</v>
+      </c>
+      <c r="P2" t="n">
         <v>100</v>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="S2" t="n">
         <v>1964</v>
       </c>
-      <c r="R2" t="n">
+      <c r="T2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="S2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>1735</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="W2" t="b">
-        <v>1</v>
-      </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="Y2" t="n">
+      <c r="AA2" t="n">
         <v>1964</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AB2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AA2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="AD2" t="n">
+      <c r="AF2" t="n">
         <v>1964</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AG2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AF2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="AI2" t="n">
+      <c r="AK2" t="n">
         <v>1735</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AL2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="AK2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AM2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="AN2" t="n">
+      <c r="AP2" t="n">
         <v>1964</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AQ2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AP2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
+      <c r="AR2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>-3.920570264765784</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AU2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AT2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
       <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AW2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>1.8777933430313</v>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>-7.289262588969585</v>
       </c>
     </row>
     <row r="3">
@@ -896,141 +912,147 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1562.868810989135</v>
+        <v>1976.631747550089</v>
       </c>
       <c r="M3" t="n">
-        <v>239.3835359491156</v>
+        <v>278.9664495260436</v>
       </c>
       <c r="N3" t="n">
+        <v>1612.384777577997</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1660.627198438829</v>
+      </c>
+      <c r="P3" t="n">
         <v>100</v>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="S3" t="n">
         <v>1571</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="S3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="b">
+        <v>1</v>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>-773</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="W3" t="b">
-        <v>1</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="inlineStr">
         <is>
           <t>[1, 8, 2, 1]</t>
         </is>
       </c>
-      <c r="Y3" t="n">
+      <c r="AA3" t="n">
         <v>-669</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AB3" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="AA3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="AD3" t="n">
+      <c r="AF3" t="n">
         <v>1571</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AG3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AF3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AH3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="AI3" t="n">
+      <c r="AK3" t="n">
         <v>-773</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AL3" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AK3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AM3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="AN3" t="n">
+      <c r="AP3" t="n">
         <v>1571</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AQ3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AP3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
+      <c r="AR3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
         <v>-5.410566518141311</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AU3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="AV3" t="n">
         <v>142.5843411839593</v>
       </c>
-      <c r="AU3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV3" t="n">
+      <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX3" t="n">
-        <v>0.5175804589983942</v>
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>-25.81997119987834</v>
       </c>
     </row>
     <row r="4">
@@ -1072,141 +1094,147 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2819.378375257139</v>
+        <v>2466.607924425859</v>
       </c>
       <c r="M4" t="n">
-        <v>205.3565369082927</v>
+        <v>338.6725224593831</v>
       </c>
       <c r="N4" t="n">
+        <v>2006.351962460336</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2002.765712135173</v>
+      </c>
+      <c r="P4" t="n">
         <v>100</v>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="S4" t="n">
         <v>2806</v>
       </c>
-      <c r="R4" t="n">
+      <c r="T4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="S4" t="b">
-        <v>1</v>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="b">
+        <v>1</v>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>976</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="W4" t="b">
-        <v>1</v>
-      </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="Y4" t="n">
+      <c r="AA4" t="n">
         <v>2806</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AB4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AA4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="AD4" t="n">
+      <c r="AF4" t="n">
         <v>2806</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AG4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AF4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AH4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AI4" t="n">
+      <c r="AK4" t="n">
         <v>976</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AL4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="AK4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
+      <c r="AM4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="AN4" t="n">
+      <c r="AP4" t="n">
         <v>2806</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="AQ4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AP4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="n">
+      <c r="AR4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
         <v>11.40413399857448</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="AU4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
       <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>-0.4767774503613308</v>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>12.09522721219318</v>
       </c>
     </row>
     <row r="5">
@@ -1248,130 +1276,130 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>1274.754116106943</v>
+        <v>1403.435230375287</v>
       </c>
       <c r="M5" t="n">
-        <v>229.4779984606443</v>
+        <v>312.7132147007493</v>
       </c>
       <c r="N5" t="n">
+        <v>958.5223937685921</v>
+      </c>
+      <c r="O5" t="n">
+        <v>985.9282551916779</v>
+      </c>
+      <c r="P5" t="n">
         <v>100</v>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="S5" t="n">
         <v>1281</v>
       </c>
-      <c r="R5" t="n">
+      <c r="T5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="S5" t="b">
-        <v>1</v>
-      </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="U5" t="n">
+      <c r="W5" t="n">
         <v>1281</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="W5" t="b">
-        <v>1</v>
-      </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="Y5" t="n">
+      <c r="AA5" t="n">
         <v>1281</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AB5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AA5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AC5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AD5" t="n">
+      <c r="AF5" t="n">
         <v>1281</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AG5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AF5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AH5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AI5" t="n">
+      <c r="AK5" t="n">
         <v>1281</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AL5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AK5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
+      <c r="AM5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AN5" t="n">
+      <c r="AP5" t="n">
         <v>1281</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AQ5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AP5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
+      <c r="AR5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
         <v>-4.918032786885246</v>
       </c>
-      <c r="AS5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>0</v>
-      </c>
       <c r="AU5" t="n">
         <v>0</v>
       </c>
@@ -1382,7 +1410,13 @@
         <v>0</v>
       </c>
       <c r="AX5" t="n">
-        <v>0.4875787582402206</v>
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>-9.557785353262034</v>
       </c>
     </row>
     <row r="6">
@@ -1424,130 +1458,130 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>1106.777517792156</v>
+        <v>1402.47343511468</v>
       </c>
       <c r="M6" t="n">
-        <v>227.9874804161272</v>
+        <v>280.386931646636</v>
       </c>
       <c r="N6" t="n">
+        <v>1024.707729684514</v>
+      </c>
+      <c r="O6" t="n">
+        <v>1109.482474335595</v>
+      </c>
+      <c r="P6" t="n">
         <v>100</v>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="S6" t="n">
         <v>1080</v>
       </c>
-      <c r="R6" t="n">
+      <c r="T6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="S6" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="b">
+        <v>1</v>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>1080</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="W6" t="b">
-        <v>1</v>
-      </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="Y6" t="n">
+      <c r="AA6" t="n">
         <v>1080</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AB6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AA6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AC6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AD6" t="n">
+      <c r="AF6" t="n">
         <v>1080</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AG6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AF6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AI6" t="n">
+      <c r="AK6" t="n">
         <v>1080</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AL6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AK6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM6" t="inlineStr">
+      <c r="AM6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AN6" t="n">
+      <c r="AP6" t="n">
         <v>1080</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AQ6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AP6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
+      <c r="AR6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
         <v>-18.61111111111111</v>
       </c>
-      <c r="AS6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>0</v>
-      </c>
       <c r="AU6" t="n">
         <v>0</v>
       </c>
@@ -1558,7 +1592,13 @@
         <v>0</v>
       </c>
       <c r="AX6" t="n">
-        <v>-2.479399795570021</v>
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>-29.85865139950737</v>
       </c>
     </row>
     <row r="7">
@@ -1600,130 +1640,130 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>733.5806640148237</v>
+        <v>784.9466263126574</v>
       </c>
       <c r="M7" t="n">
-        <v>167.5705297236776</v>
+        <v>372.961520330355</v>
       </c>
       <c r="N7" t="n">
+        <v>263.0094503251535</v>
+      </c>
+      <c r="O7" t="n">
+        <v>300.0046004505125</v>
+      </c>
+      <c r="P7" t="n">
         <v>100</v>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="S7" t="n">
         <v>774</v>
       </c>
-      <c r="R7" t="n">
+      <c r="T7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="S7" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="b">
+        <v>1</v>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>774</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="W7" t="b">
-        <v>1</v>
-      </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="Y7" t="n">
+      <c r="AA7" t="n">
         <v>774</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AB7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AA7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AC7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AD7" t="n">
+      <c r="AF7" t="n">
         <v>774</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AG7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AF7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AH7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AI7" t="n">
+      <c r="AK7" t="n">
         <v>774</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AL7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AK7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM7" t="inlineStr">
+      <c r="AM7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AN7" t="n">
+      <c r="AP7" t="n">
         <v>774</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AQ7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AP7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="n">
+      <c r="AR7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
         <v>-0.9043927648578811</v>
       </c>
-      <c r="AS7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>0</v>
-      </c>
       <c r="AU7" t="n">
         <v>0</v>
       </c>
@@ -1734,7 +1774,13 @@
         <v>0</v>
       </c>
       <c r="AX7" t="n">
-        <v>5.222136432193321</v>
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>-1.41429280525289</v>
       </c>
     </row>
     <row r="8">
@@ -1776,130 +1822,130 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>1992.088721972067</v>
+        <v>2108.289215230296</v>
       </c>
       <c r="M8" t="n">
-        <v>218.4144072876398</v>
+        <v>284.2228643517807</v>
       </c>
       <c r="N8" t="n">
+        <v>1749.750460769153</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1802.007824700107</v>
+      </c>
+      <c r="P8" t="n">
         <v>100</v>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="S8" t="n">
         <v>1964</v>
       </c>
-      <c r="R8" t="n">
+      <c r="T8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="S8" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="b">
+        <v>1</v>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="U8" t="n">
+      <c r="W8" t="n">
         <v>1964</v>
       </c>
-      <c r="V8" t="n">
+      <c r="X8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="W8" t="b">
-        <v>1</v>
-      </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="Y8" t="n">
+      <c r="AA8" t="n">
         <v>1964</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AB8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AA8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AC8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="AD8" t="n">
+      <c r="AF8" t="n">
         <v>1964</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AG8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AF8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
+      <c r="AH8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="AI8" t="n">
+      <c r="AK8" t="n">
         <v>1964</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AL8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AK8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AM8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="AN8" t="n">
+      <c r="AP8" t="n">
         <v>1964</v>
       </c>
-      <c r="AO8" t="n">
+      <c r="AQ8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AP8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="n">
+      <c r="AR8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
         <v>-2.90224032586558</v>
       </c>
-      <c r="AS8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>0</v>
-      </c>
       <c r="AU8" t="n">
         <v>0</v>
       </c>
@@ -1910,7 +1956,13 @@
         <v>0</v>
       </c>
       <c r="AX8" t="n">
-        <v>-1.430179326479995</v>
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>-7.34670138647129</v>
       </c>
     </row>
     <row r="9">
@@ -1952,129 +2004,129 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>2773.479890320478</v>
+        <v>2421.27299129609</v>
       </c>
       <c r="M9" t="n">
-        <v>242.7141642794886</v>
+        <v>296.8948967168763</v>
       </c>
       <c r="N9" t="n">
+        <v>2013.065797322877</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2021.299320208423</v>
+      </c>
+      <c r="P9" t="n">
         <v>100</v>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="S9" t="n">
         <v>2794</v>
       </c>
-      <c r="R9" t="n">
+      <c r="T9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="S9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="b">
+        <v>1</v>
+      </c>
+      <c r="V9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="U9" t="n">
+      <c r="W9" t="n">
         <v>2634</v>
       </c>
-      <c r="V9" t="n">
+      <c r="X9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="W9" t="b">
-        <v>1</v>
-      </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="Y9" t="n">
+      <c r="AA9" t="n">
         <v>2634</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AB9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AA9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AC9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="AD9" t="n">
+      <c r="AF9" t="n">
         <v>2634</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AG9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AF9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
+      <c r="AH9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="AI9" t="n">
+      <c r="AK9" t="n">
         <v>2634</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AL9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AK9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM9" t="inlineStr">
+      <c r="AM9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="AN9" t="n">
+      <c r="AP9" t="n">
         <v>2634</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="AQ9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="AP9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR9" t="n">
+      <c r="AR9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
         <v>18.00286327845383</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>5.72655690765927</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>5.72655690765927</v>
       </c>
       <c r="AU9" t="n">
         <v>5.72655690765927</v>
@@ -2086,7 +2138,13 @@
         <v>5.72655690765927</v>
       </c>
       <c r="AX9" t="n">
-        <v>0.7344348489449604</v>
+        <v>5.72655690765927</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>5.72655690765927</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>13.34026516477846</v>
       </c>
     </row>
     <row r="10">
@@ -2128,130 +2186,130 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1801.844142827736</v>
+        <v>1765.19534268021</v>
       </c>
       <c r="M10" t="n">
-        <v>231.3565177255371</v>
+        <v>349.5752485625928</v>
       </c>
       <c r="N10" t="n">
+        <v>1300.654602481184</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1362.108056943827</v>
+      </c>
+      <c r="P10" t="n">
         <v>100</v>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="Q10" t="n">
+      <c r="S10" t="n">
         <v>1874</v>
       </c>
-      <c r="R10" t="n">
+      <c r="T10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="S10" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="b">
+        <v>1</v>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="U10" t="n">
+      <c r="W10" t="n">
         <v>1874</v>
       </c>
-      <c r="V10" t="n">
+      <c r="X10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="W10" t="b">
-        <v>1</v>
-      </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="Y10" t="n">
+      <c r="AA10" t="n">
         <v>1874</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AB10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AA10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AC10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="AD10" t="n">
+      <c r="AF10" t="n">
         <v>1874</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AG10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AF10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AH10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="AI10" t="n">
+      <c r="AK10" t="n">
         <v>1874</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AL10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AK10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
+      <c r="AM10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="AN10" t="n">
+      <c r="AP10" t="n">
         <v>1874</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="AQ10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="AP10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ10" t="n">
+      <c r="AR10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS10" t="n">
         <v>1.387406616862326</v>
       </c>
-      <c r="AR10" t="n">
+      <c r="AT10" t="n">
         <v>8.911419423692637</v>
       </c>
-      <c r="AS10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>0</v>
-      </c>
       <c r="AU10" t="n">
         <v>0</v>
       </c>
@@ -2262,7 +2320,13 @@
         <v>0</v>
       </c>
       <c r="AX10" t="n">
-        <v>3.850365911006627</v>
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>5.806011596573655</v>
       </c>
     </row>
     <row r="11">
@@ -2304,123 +2368,123 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>-4050.96728546096</v>
+        <v>-3965.922300613382</v>
       </c>
       <c r="M11" t="n">
-        <v>235.0732453317911</v>
+        <v>317.5167484036342</v>
       </c>
       <c r="N11" t="n">
+        <v>-4396.568462825113</v>
+      </c>
+      <c r="O11" t="n">
+        <v>-4371.169340685334</v>
+      </c>
+      <c r="P11" t="n">
         <v>100</v>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="Q11" t="n">
+      <c r="S11" t="n">
         <v>-4042</v>
       </c>
-      <c r="R11" t="n">
+      <c r="T11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="S11" t="b">
-        <v>1</v>
-      </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="b">
+        <v>1</v>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="U11" t="n">
+      <c r="W11" t="n">
         <v>-4042</v>
       </c>
-      <c r="V11" t="n">
+      <c r="X11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="W11" t="b">
-        <v>1</v>
-      </c>
-      <c r="X11" t="inlineStr">
+      <c r="Y11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="Y11" t="n">
+      <c r="AA11" t="n">
         <v>-4042</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AB11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AA11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AC11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AD11" t="n">
+      <c r="AF11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AG11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AF11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AH11" t="inlineStr">
+      <c r="AH11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AI11" t="n">
+      <c r="AK11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AL11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AK11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AM11" t="inlineStr">
+      <c r="AM11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AN11" t="n">
+      <c r="AP11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AO11" t="n">
+      <c r="AQ11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AP11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>0</v>
+      <c r="AR11" t="b">
+        <v>1</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2438,7 +2502,13 @@
         <v>0</v>
       </c>
       <c r="AX11" t="n">
-        <v>0.2218526833488442</v>
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>-1.882179598877249</v>
       </c>
     </row>
   </sheetData>
@@ -2548,13 +2618,13 @@
         <v>1190.6</v>
       </c>
       <c r="J2" t="n">
-        <v>1021.136117458344</v>
+        <v>1007.758345603943</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8525385863352319</v>
+        <v>-5.192734035867348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adición Rolling Horizon Greedy
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_stochastic_sigma10%_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:AY11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,22 +537,22 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Route</t>
+          <t>RH-Greedy Route</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Reward</t>
+          <t>RH-Greedy Reward</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Duration</t>
+          <t>RH-Greedy Duration</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Valid</t>
+          <t>RH-Greedy Valid</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -662,30 +662,25 @@
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Gap (%)</t>
+          <t>2Opt Gap (%)</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>2Opt Gap (%)</t>
+          <t>GA Gap (%)</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>GA Gap (%)</t>
+          <t>LNS Gap (%)</t>
         </is>
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>LNS Gap (%)</t>
+          <t>HGA-LNS Gap (%)</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>HGA-LNS Gap (%)</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>DRL Stoch Gap (%)</t>
         </is>
@@ -769,7 +764,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>1735</v>
+        <v>1828</v>
       </c>
       <c r="X2" t="n">
         <v>55.44764714720212</v>
@@ -855,21 +850,18 @@
         <v>-3.920570264765784</v>
       </c>
       <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AV2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW2" t="n">
-        <v>0</v>
-      </c>
       <c r="AX2" t="n">
-        <v>11.65987780040733</v>
+        <v>0</v>
       </c>
       <c r="AY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ2" t="n">
         <v>-7.289262588969585</v>
       </c>
     </row>
@@ -912,16 +904,16 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
-        <v>1976.631747550089</v>
+        <v>1958.254797785167</v>
       </c>
       <c r="M3" t="n">
-        <v>278.9664495260436</v>
+        <v>295.0111175404787</v>
       </c>
       <c r="N3" t="n">
-        <v>1612.384777577997</v>
+        <v>1551.216718109133</v>
       </c>
       <c r="O3" t="n">
-        <v>1660.627198438829</v>
+        <v>1585.305496162799</v>
       </c>
       <c r="P3" t="n">
         <v>100</v>
@@ -951,7 +943,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>-773</v>
+        <v>1164</v>
       </c>
       <c r="X3" t="n">
         <v>70.15987690240341</v>
@@ -1037,22 +1029,19 @@
         <v>-5.410566518141311</v>
       </c>
       <c r="AU3" t="n">
+        <v>142.5843411839593</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AV3" t="n">
-        <v>142.5843411839593</v>
-      </c>
-      <c r="AW3" t="n">
-        <v>0</v>
-      </c>
       <c r="AX3" t="n">
-        <v>149.2043284532145</v>
+        <v>0</v>
       </c>
       <c r="AY3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ3" t="n">
-        <v>-25.81997119987834</v>
+        <v>-24.65020991630596</v>
       </c>
     </row>
     <row r="4">
@@ -1094,16 +1083,16 @@
         <v>1</v>
       </c>
       <c r="L4" t="n">
-        <v>2466.607924425859</v>
+        <v>2525.848469461252</v>
       </c>
       <c r="M4" t="n">
-        <v>338.6725224593831</v>
+        <v>304.1598535735931</v>
       </c>
       <c r="N4" t="n">
-        <v>2006.351962460336</v>
+        <v>2095.729199581938</v>
       </c>
       <c r="O4" t="n">
-        <v>2002.765712135173</v>
+        <v>2176.917710353405</v>
       </c>
       <c r="P4" t="n">
         <v>100</v>
@@ -1133,7 +1122,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>976</v>
+        <v>-1221</v>
       </c>
       <c r="X4" t="n">
         <v>72.45471862628276</v>
@@ -1219,22 +1208,19 @@
         <v>11.40413399857448</v>
       </c>
       <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AV4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>0</v>
-      </c>
       <c r="AX4" t="n">
-        <v>65.21739130434783</v>
+        <v>0</v>
       </c>
       <c r="AY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>12.09522721219318</v>
+        <v>9.98401748178004</v>
       </c>
     </row>
     <row r="5">
@@ -1276,16 +1262,16 @@
         <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>1403.435230375287</v>
+        <v>1364.991704707495</v>
       </c>
       <c r="M5" t="n">
-        <v>312.7132147007493</v>
+        <v>316.2318162212319</v>
       </c>
       <c r="N5" t="n">
-        <v>958.5223937685921</v>
+        <v>941.6863114502618</v>
       </c>
       <c r="O5" t="n">
-        <v>985.9282551916779</v>
+        <v>953.8339862755829</v>
       </c>
       <c r="P5" t="n">
         <v>100</v>
@@ -1315,7 +1301,7 @@
         </is>
       </c>
       <c r="W5" t="n">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="X5" t="n">
         <v>40.68356024804761</v>
@@ -1413,10 +1399,7 @@
         <v>0</v>
       </c>
       <c r="AY5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ5" t="n">
-        <v>-9.557785353262034</v>
+        <v>-6.556729485362575</v>
       </c>
     </row>
     <row r="6">
@@ -1458,16 +1441,16 @@
         <v>1</v>
       </c>
       <c r="L6" t="n">
-        <v>1402.47343511468</v>
+        <v>1339.326543224434</v>
       </c>
       <c r="M6" t="n">
-        <v>280.386931646636</v>
+        <v>278.6521081997284</v>
       </c>
       <c r="N6" t="n">
-        <v>1024.707729684514</v>
+        <v>948.0993223256107</v>
       </c>
       <c r="O6" t="n">
-        <v>1109.482474335595</v>
+        <v>976.709692392324</v>
       </c>
       <c r="P6" t="n">
         <v>100</v>
@@ -1595,10 +1578,7 @@
         <v>0</v>
       </c>
       <c r="AY6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ6" t="n">
-        <v>-29.85865139950737</v>
+        <v>-24.01171696522536</v>
       </c>
     </row>
     <row r="7">
@@ -1640,16 +1620,16 @@
         <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>784.9466263126574</v>
+        <v>803.5230128086782</v>
       </c>
       <c r="M7" t="n">
-        <v>372.961520330355</v>
+        <v>305.9753186426074</v>
       </c>
       <c r="N7" t="n">
-        <v>263.0094503251535</v>
+        <v>355.2752018313509</v>
       </c>
       <c r="O7" t="n">
-        <v>300.0046004505125</v>
+        <v>311.3467808251878</v>
       </c>
       <c r="P7" t="n">
         <v>100</v>
@@ -1777,10 +1757,7 @@
         <v>0</v>
       </c>
       <c r="AY7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ7" t="n">
-        <v>-1.41429280525289</v>
+        <v>-3.814342740139307</v>
       </c>
     </row>
     <row r="8">
@@ -1822,16 +1799,16 @@
         <v>1</v>
       </c>
       <c r="L8" t="n">
-        <v>2108.289215230296</v>
+        <v>2136.952071062804</v>
       </c>
       <c r="M8" t="n">
-        <v>284.2228643517807</v>
+        <v>285.0947597178829</v>
       </c>
       <c r="N8" t="n">
-        <v>1749.750460769153</v>
+        <v>1726.60882161935</v>
       </c>
       <c r="O8" t="n">
-        <v>1802.007824700107</v>
+        <v>1778.722862706227</v>
       </c>
       <c r="P8" t="n">
         <v>100</v>
@@ -1861,7 +1838,7 @@
         </is>
       </c>
       <c r="W8" t="n">
-        <v>1964</v>
+        <v>1870</v>
       </c>
       <c r="X8" t="n">
         <v>76.7052345103569</v>
@@ -1959,10 +1936,7 @@
         <v>0</v>
       </c>
       <c r="AY8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="n">
-        <v>-7.34670138647129</v>
+        <v>-8.806113597902465</v>
       </c>
     </row>
     <row r="9">
@@ -2004,16 +1978,16 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>2421.27299129609</v>
+        <v>2477.352902108788</v>
       </c>
       <c r="M9" t="n">
-        <v>296.8948967168763</v>
+        <v>285.8549252820411</v>
       </c>
       <c r="N9" t="n">
-        <v>2013.065797322877</v>
+        <v>2110.92877063223</v>
       </c>
       <c r="O9" t="n">
-        <v>2021.299320208423</v>
+        <v>2130.365013076027</v>
       </c>
       <c r="P9" t="n">
         <v>100</v>
@@ -2043,7 +2017,7 @@
         </is>
       </c>
       <c r="W9" t="n">
-        <v>2634</v>
+        <v>1379</v>
       </c>
       <c r="X9" t="n">
         <v>76.25197526044872</v>
@@ -2141,10 +2115,7 @@
         <v>5.72655690765927</v>
       </c>
       <c r="AY9" t="n">
-        <v>5.72655690765927</v>
-      </c>
-      <c r="AZ9" t="n">
-        <v>13.34026516477846</v>
+        <v>11.33311016074487</v>
       </c>
     </row>
     <row r="10">
@@ -2186,16 +2157,16 @@
         <v>1</v>
       </c>
       <c r="L10" t="n">
-        <v>1765.19534268021</v>
+        <v>1752.184723367529</v>
       </c>
       <c r="M10" t="n">
-        <v>349.5752485625928</v>
+        <v>310.8838567121231</v>
       </c>
       <c r="N10" t="n">
-        <v>1300.654602481184</v>
+        <v>1357.512825901907</v>
       </c>
       <c r="O10" t="n">
-        <v>1362.108056943827</v>
+        <v>1402.982723184966</v>
       </c>
       <c r="P10" t="n">
         <v>100</v>
@@ -2225,7 +2196,7 @@
         </is>
       </c>
       <c r="W10" t="n">
-        <v>1874</v>
+        <v>1500</v>
       </c>
       <c r="X10" t="n">
         <v>70.15987690240343</v>
@@ -2323,10 +2294,7 @@
         <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ10" t="n">
-        <v>5.806011596573655</v>
+        <v>6.500281570569427</v>
       </c>
     </row>
     <row r="11">
@@ -2368,16 +2336,16 @@
         <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>-3965.922300613382</v>
+        <v>-3952.758442001685</v>
       </c>
       <c r="M11" t="n">
-        <v>317.5167484036342</v>
+        <v>301.0450800954807</v>
       </c>
       <c r="N11" t="n">
-        <v>-4396.568462825113</v>
+        <v>-4394.284291856744</v>
       </c>
       <c r="O11" t="n">
-        <v>-4371.169340685334</v>
+        <v>-4339.799404999199</v>
       </c>
       <c r="P11" t="n">
         <v>100</v>
@@ -2505,10 +2473,7 @@
         <v>0</v>
       </c>
       <c r="AY11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ11" t="n">
-        <v>-1.882179598877249</v>
+        <v>-2.207856457157727</v>
       </c>
     </row>
   </sheetData>
@@ -2548,27 +2513,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Heuristic Avg</t>
+          <t>2Opt Avg</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>2Opt Avg</t>
+          <t>GA Avg</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>GA Avg</t>
+          <t>LNS Avg</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LNS Avg</t>
+          <t>HGA-LNS Avg</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Avg</t>
+          <t>RH-Greedy Avg</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -2603,28 +2568,28 @@
         <v>1204</v>
       </c>
       <c r="E2" t="n">
+        <v>966.6</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1190.6</v>
+      </c>
+      <c r="G2" t="n">
         <v>750.3</v>
       </c>
-      <c r="F2" t="n">
-        <v>966.6</v>
-      </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1190.6</v>
       </c>
-      <c r="H2" t="n">
-        <v>750.3</v>
-      </c>
       <c r="I2" t="n">
-        <v>1190.6</v>
+        <v>561.4</v>
       </c>
       <c r="J2" t="n">
-        <v>1007.758345603943</v>
+        <v>994.5328507423401</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>
       </c>
       <c r="L2" t="n">
-        <v>-5.192734035867348</v>
+        <v>-4.951882253796864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>